<commit_message>
feat(W3.4): portfolio home — pipeline, 5D/SDG heat-map, deadlines, review queue
- impact/portfolio_home.py + portfolio_home.html.j2 on the shared design system
- web: Reports -> Open portfolio home (/api/v1/chat/portfolio/view), newest report per company
- demo/portfolio_home.html linked from the gallery; axe/responsive QA coverage
- README screenshots (chat analyze card, report viewer, portfolio home); Wave 3 status

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo/brightpath_finance/brightpath_finance_data.xlsx
+++ b/demo/brightpath_finance/brightpath_finance_data.xlsx
@@ -525,7 +525,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-06T08:53:40Z</t>
+          <t>2026-10-06T10:36:51Z</t>
         </is>
       </c>
     </row>
@@ -2067,7 +2067,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-10-06T08:53:40Z</t>
+          <t>2026-10-06T10:36:51Z</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>

</xml_diff>

<commit_message>
release: 0.17.0 "Trusted, Effortless & Beautiful"
- version 0.17.0 everywhere (pyproject is the single source; CLI and /health read it);
  CHANGELOG [0.17.0] consolidates roadmap v7 Waves 0-5 + follow-ups; AGENTS.md synced
- methodology 1.1.0: per-SDG core metric sets rebuilt (half the IDs pointed at the
  wrong IRIS+ metric), own-footprint metrics and footprint-only sentences no longer
  drive SDG 13; guard tests for every core-set entry
- engagement view: completion percentages scaled, 'no checklist' state, no date wrapping;
  visual QA covers it
- demo regenerated (adds engagements.html); all README/demo screenshots recaptured,
  web shots reproducible via capture_screenshots.py --seed-web; README updated (849 lines)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo/brightpath_finance/brightpath_finance_data.xlsx
+++ b/demo/brightpath_finance/brightpath_finance_data.xlsx
@@ -13,16 +13,18 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gap Analysis" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Claims" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All figures" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI provenance" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$3:$B$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$3:$B$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'5 Dimensions'!$A$1:$E$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'SDG Alignment'!$A$1:$G$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Gap Analysis'!$A$1:$F$18</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Claims'!$A$1:$E$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'All figures'!$A$1:$G$48</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Methodology'!$A$1:$B$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Claims'!$A$1:$F$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'All figures'!$A$1:$G$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'AI provenance'!$A$13:$F$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Methodology'!$A$1:$B$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -455,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -525,7 +527,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-06T10:36:51Z</t>
+          <t>2026-10-07T00:37:40Z</t>
         </is>
       </c>
     </row>
@@ -572,7 +574,7 @@
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="12">
@@ -594,7 +596,7 @@
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>58.9</v>
+        <v>57.1</v>
       </c>
     </row>
     <row r="14">
@@ -614,23 +616,59 @@
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>AI disclosure</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Automated analysis: produced by rules and a deterministic scoring model; no generative AI was used. 3 of 21 scores are estimated from document text rather than reported metrics. Review before relying on it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Methodology version</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>1.1.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Methodology config hash</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>8fabf9b5a7e2</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>Export schema</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>1.0</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:B16"/>
+  <autoFilter ref="A3:B19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -685,7 +723,7 @@
         </is>
       </c>
       <c r="B2" s="4" t="n">
-        <v>1.8</v>
+        <v>1.5</v>
       </c>
       <c r="C2" t="n">
         <v>2</v>
@@ -769,7 +807,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="C6" t="n">
         <v>0</v>
@@ -790,7 +828,7 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -818,7 +856,7 @@
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
     <col width="41" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -861,19 +899,19 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Climate Action</t>
+          <t>No Poverty</t>
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>66</v>
+        <v>42.7</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -883,26 +921,26 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>OI1479, OI4112, PI4060</t>
+          <t>PI4060</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>13.1, 13.2</t>
+          <t>1.4, 1.5</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Reduced Inequalities</t>
+          <t>Zero Hunger</t>
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>41.9</v>
+        <v>42.7</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -916,26 +954,26 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>OI1571, OI6213, PI4060</t>
+          <t>PI4060</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>10.1, 10.2, 10.3, 10.c</t>
+          <t>2.1, 2.3, 2.4</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Zero Hunger</t>
+          <t>Gender Equality</t>
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>41</v>
+        <v>37.8</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -949,26 +987,26 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>PI4060</t>
+          <t>OI1571, OI6213</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2.1, 2.3, 2.4</t>
+          <t>5.1, 5.2, 5.5</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>No Poverty</t>
+          <t>Decent Work and Economic Growth</t>
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>39.8</v>
+        <v>37.3</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -982,26 +1020,26 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>PI4060</t>
+          <t>OI6213, OI8869</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>1.4, 1.5</t>
+          <t>8.1, 8.10, 8.2, 8.3, 8.5, 8.6, 8.7, 8.8</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Gender Equality</t>
+          <t>Industry, Innovation and Infrastructure</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>39.5</v>
+        <v>35.5</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1015,26 +1053,26 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>OI1571, OI6213</t>
+          <t>OI8869, PI4060</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>5.1, 5.2, 5.5</t>
+          <t>9.1, 9.3</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Decent Work and Economic Growth</t>
+          <t>Reduced Inequalities</t>
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>39.5</v>
+        <v>35.2</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1048,26 +1086,26 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>OI1571, OI6213, OI8869, PI4060</t>
+          <t>PI4060</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>8.1, 8.10, 8.2, 8.3, 8.5, 8.6, 8.7, 8.8</t>
+          <t>10.1, 10.2, 10.3, 10.c</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Industry, Innovation and Infrastructure</t>
+          <t>Clean Water and Sanitation</t>
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>38.5</v>
+        <v>28</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1076,31 +1114,31 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>OI8869, PI4060</t>
+          <t>PI4060</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>9.1, 9.3</t>
+          <t>6.1, 6.2, 6.4</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Clean Water and Sanitation</t>
+          <t>Good Health and Well-being</t>
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>32</v>
+        <v>27.7</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1119,21 +1157,21 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>6.1, 6.2, 6.4</t>
+          <t>3.3, 3.4, 3.5, 3.7, 3.8, 3.9</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Affordable and Clean Energy</t>
+          <t>Peace, Justice and Strong Institutions</t>
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>32</v>
+        <v>27.5</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1142,31 +1180,23 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>PI4060</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>7.1</t>
-        </is>
-      </c>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Good Health and Well-being</t>
+          <t>Affordable and Clean Energy</t>
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>24.8</v>
+        <v>25</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1178,24 +1208,20 @@
           <t>no</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>PI4060</t>
-        </is>
-      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>3.3, 3.4, 3.5, 3.7, 3.8, 3.9</t>
+          <t>7.1</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Peace, Justice and Strong Institutions</t>
+          <t>Life on Land</t>
         </is>
       </c>
       <c r="C12" s="4" t="n">
@@ -1208,7 +1234,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
@@ -1216,15 +1242,15 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Quality Education</t>
+          <t>Climate Action</t>
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>20</v>
+        <v>20.3</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1238,22 +1264,22 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>PI4060</t>
+          <t>OI1479, OI4112</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>4.1, 4.2, 4.3, 4.4, 4.5, 4.a</t>
+          <t>13.1, 13.2</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Sustainable Cities and Communities</t>
+          <t>Quality Education</t>
         </is>
       </c>
       <c r="C14" s="4" t="n">
@@ -1276,22 +1302,22 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>11.1, 11.2, 11.3, 11.5, 11.6</t>
+          <t>4.1, 4.2, 4.3, 4.4, 4.5, 4.a</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Sustainable Cities and Communities</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Life on Land</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="n">
-        <v>17.5</v>
-      </c>
       <c r="D15" t="inlineStr">
         <is>
           <t>low</t>
@@ -1303,7 +1329,11 @@
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>11.1, 11.2, 11.3, 11.5, 11.6</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1315,7 +1345,7 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1344,7 +1374,7 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1853,7 +1883,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1861,6 +1891,7 @@
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1889,6 +1920,11 @@
           <t>Mapped metrics</t>
         </is>
       </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Extracted by</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1912,6 +1948,11 @@
           <t>PI4060</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>regex</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1919,9 +1960,9 @@
           <t>outcome</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Revenue grew 32% last year (FP4761: 32%).</t>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>We employ 180 permanent staff (OI8869: 180), including 85 women (OI6213: 85) and 12 female managers (OI1571: 12).</t>
         </is>
       </c>
       <c r="C3" s="6" t="n">
@@ -1930,7 +1971,16 @@
       <c r="D3" s="7" t="n">
         <v>0.3</v>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>OI8869</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>regex</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1940,7 +1990,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Portfolio at risk over 30 days is 3.1%.</t>
+          <t>Revenue grew 32% last year (FP4761: 32%).</t>
         </is>
       </c>
       <c r="C4" s="6" t="n">
@@ -1950,6 +2000,11 @@
         <v>0.3</v>
       </c>
       <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>regex</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1957,9 +2012,9 @@
           <t>outcome</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Our own footprint is 120 tCO2e (OI1479: 120 tCO2e), of which 80 tCO2e are direct Scope 1 emissions (OI4112: 80 tCO2e).</t>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Portfolio at risk over 30 days is 3.1%.</t>
         </is>
       </c>
       <c r="C5" s="6" t="n">
@@ -1968,14 +2023,43 @@
       <c r="D5" s="7" t="n">
         <v>0.3</v>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>OI1479</t>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>regex</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>outcome</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Our own footprint is 120 tCO2e (OI1479: 120 tCO2e), of which 80 tCO2e are direct Scope 1 emissions (OI4112: 80 tCO2e).</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>OI1479, OI4112</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>regex</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E5"/>
+  <autoFilter ref="A1:F6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1986,7 +2070,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2067,7 +2151,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-10-06T10:36:51Z</t>
+          <t>2026-10-07T00:37:40Z</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -2076,68 +2160,44 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>5D</t>
+          <t>Company</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Overall Grade</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>1.8/5.0</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="F4" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>score</t>
-        </is>
-      </c>
+          <t>AI disclosure</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Automated analysis: produced by rules and a deterministic scoring model; no generative AI was used. 3 of 21 scores are estimated from document text rather than reported metrics. Review before relying on it.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>5D</t>
+          <t>Company</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>Methodology</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1.8/5.0</t>
+          <t>1.1.0</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Reporting 2 metrics (0 theme-specific, 14 available)</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="F5" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>score</t>
-        </is>
-      </c>
+          <t>config 8fabf9b5a7e2</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2147,21 +2207,21 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Who</t>
+          <t>Overall Grade</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2.5/5.0</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Reporting 5 metrics (0 theme-specific, 6 available)</t>
+          <t>1.7/5.0</t>
         </is>
       </c>
       <c r="E6" s="5" t="n">
-        <v>2.5</v>
+        <v>1.7</v>
       </c>
       <c r="F6" s="6" t="n">
         <v>5</v>
@@ -2180,21 +2240,21 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>How Much</t>
+          <t>What</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>1.8/5.0</t>
+          <t>1.5/5.0</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Scale=1.8, Depth=1.8, Duration=1.8</t>
+          <t>Reporting 2 metrics (0 theme-specific, 14 available)</t>
         </is>
       </c>
       <c r="E7" s="5" t="n">
-        <v>1.8</v>
+        <v>1.5</v>
       </c>
       <c r="F7" s="6" t="n">
         <v>5</v>
@@ -2213,21 +2273,21 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Contribution</t>
+          <t>Who</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1.5/5.0</t>
+          <t>2.5/5.0</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Depth=1.5, Duration=1.5</t>
+          <t>Reporting 5 metrics (0 theme-specific, 6 available)</t>
         </is>
       </c>
       <c r="E8" s="5" t="n">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
       <c r="F8" s="6" t="n">
         <v>5</v>
@@ -2246,21 +2306,21 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Risk</t>
+          <t>How Much</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1.5/5.0</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>Estimated from sector/description (4 metrics available to track)</t>
+          <t>1.8/5.0</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Scale=1.8, Depth=1.8, Duration=1.8</t>
         </is>
       </c>
       <c r="E9" s="5" t="n">
-        <v>1.5</v>
+        <v>1.8</v>
       </c>
       <c r="F9" s="6" t="n">
         <v>5</v>
@@ -2274,29 +2334,29 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SDG</t>
+          <t>5D</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>SDG 13</t>
+          <t>Contribution</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>66.0/100</t>
+          <t>1.5/5.0</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>high | metrics: OI1479,OI4112,PI4060</t>
+          <t>Depth=1.5, Duration=1.5</t>
         </is>
       </c>
       <c r="E10" s="5" t="n">
-        <v>66</v>
+        <v>1.5</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -2307,29 +2367,29 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SDG</t>
+          <t>5D</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>SDG 10</t>
+          <t>Risk</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>41.9/100</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>medium | metrics: OI1571,OI6213,PI4060</t>
+          <t>1.2/5.0</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Estimated from sector/description (4 metrics available to track)</t>
         </is>
       </c>
       <c r="E11" s="5" t="n">
-        <v>41.9</v>
+        <v>1.2</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -2345,12 +2405,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>SDG 2</t>
+          <t>SDG 1</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>41.0/100</t>
+          <t>42.7/100</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -2359,7 +2419,7 @@
         </is>
       </c>
       <c r="E12" s="5" t="n">
-        <v>41</v>
+        <v>42.7</v>
       </c>
       <c r="F12" s="6" t="n">
         <v>100</v>
@@ -2378,12 +2438,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>SDG 1</t>
+          <t>SDG 2</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>39.8/100</t>
+          <t>42.7/100</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2392,7 +2452,7 @@
         </is>
       </c>
       <c r="E13" s="5" t="n">
-        <v>39.8</v>
+        <v>42.7</v>
       </c>
       <c r="F13" s="6" t="n">
         <v>100</v>
@@ -2416,7 +2476,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>39.5/100</t>
+          <t>37.8/100</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2425,7 +2485,7 @@
         </is>
       </c>
       <c r="E14" s="5" t="n">
-        <v>39.5</v>
+        <v>37.8</v>
       </c>
       <c r="F14" s="6" t="n">
         <v>100</v>
@@ -2449,16 +2509,16 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>39.5/100</t>
+          <t>37.3/100</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>medium | metrics: OI1571,OI6213,OI8869</t>
+          <t>medium | metrics: OI6213,OI8869</t>
         </is>
       </c>
       <c r="E15" s="5" t="n">
-        <v>39.5</v>
+        <v>37.3</v>
       </c>
       <c r="F15" s="6" t="n">
         <v>100</v>
@@ -2482,7 +2542,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>38.5/100</t>
+          <t>35.5/100</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -2491,7 +2551,7 @@
         </is>
       </c>
       <c r="E16" s="5" t="n">
-        <v>38.5</v>
+        <v>35.5</v>
       </c>
       <c r="F16" s="6" t="n">
         <v>100</v>
@@ -2510,12 +2570,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>SDG 6</t>
+          <t>SDG 10</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>32.0/100</t>
+          <t>35.2/100</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2524,7 +2584,7 @@
         </is>
       </c>
       <c r="E17" s="5" t="n">
-        <v>32</v>
+        <v>35.2</v>
       </c>
       <c r="F17" s="6" t="n">
         <v>100</v>
@@ -2543,12 +2603,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>SDG 7</t>
+          <t>SDG 6</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>32.0/100</t>
+          <t>28.0/100</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2557,7 +2617,7 @@
         </is>
       </c>
       <c r="E18" s="5" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="F18" s="6" t="n">
         <v>100</v>
@@ -2581,7 +2641,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>24.8/100</t>
+          <t>27.7/100</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2590,7 +2650,7 @@
         </is>
       </c>
       <c r="E19" s="5" t="n">
-        <v>24.8</v>
+        <v>27.7</v>
       </c>
       <c r="F19" s="6" t="n">
         <v>100</v>
@@ -2614,7 +2674,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>22.5/100</t>
+          <t>27.5/100</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2623,7 +2683,7 @@
         </is>
       </c>
       <c r="E20" s="5" t="n">
-        <v>22.5</v>
+        <v>27.5</v>
       </c>
       <c r="F20" s="6" t="n">
         <v>100</v>
@@ -2642,21 +2702,21 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>SDG 4</t>
+          <t>SDG 7</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>20.0/100</t>
+          <t>25.0/100</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>medium | metrics: PI4060</t>
+          <t xml:space="preserve">medium | metrics: </t>
         </is>
       </c>
       <c r="E21" s="5" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F21" s="6" t="n">
         <v>100</v>
@@ -2675,21 +2735,21 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>SDG 11</t>
+          <t>SDG 15</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>18.0/100</t>
+          <t>22.5/100</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>low | metrics: PI4060</t>
+          <t xml:space="preserve">medium | metrics: </t>
         </is>
       </c>
       <c r="E22" s="5" t="n">
-        <v>18</v>
+        <v>22.5</v>
       </c>
       <c r="F22" s="6" t="n">
         <v>100</v>
@@ -2708,21 +2768,21 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>SDG 15</t>
+          <t>SDG 13</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>17.5/100</t>
+          <t>20.3/100</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">low | metrics: </t>
+          <t>medium | metrics: OI1479,OI4112</t>
         </is>
       </c>
       <c r="E23" s="5" t="n">
-        <v>17.5</v>
+        <v>20.3</v>
       </c>
       <c r="F23" s="6" t="n">
         <v>100</v>
@@ -2741,21 +2801,21 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>SDG 12</t>
+          <t>SDG 4</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>10.0/100</t>
+          <t>18.0/100</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve">low | metrics: </t>
+          <t>low | metrics: PI4060</t>
         </is>
       </c>
       <c r="E24" s="5" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F24" s="6" t="n">
         <v>100</v>
@@ -2774,12 +2834,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>SDG 14</t>
+          <t>SDG 11</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>10.0/100</t>
+          <t>15.0/100</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2788,7 +2848,7 @@
         </is>
       </c>
       <c r="E25" s="5" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F25" s="6" t="n">
         <v>100</v>
@@ -2802,87 +2862,101 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Greenwashing</t>
+          <t>SDG</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Risk score</t>
+          <t>SDG 12</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>58.9/100</t>
+          <t>15.0/100</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Moderate Risk</t>
+          <t xml:space="preserve">low | metrics: </t>
         </is>
       </c>
       <c r="E26" s="5" t="n">
-        <v>58.9</v>
+        <v>15</v>
       </c>
       <c r="F26" s="6" t="n">
         <v>100</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>risk</t>
+          <t>score</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Gap</t>
+          <t>SDG</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Coverage</t>
+          <t>SDG 14</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>47.1%</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr"/>
+          <t>15.0/100</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">low | metrics: </t>
+        </is>
+      </c>
       <c r="E27" s="5" t="n">
-        <v>47.1</v>
+        <v>15</v>
       </c>
       <c r="F27" s="6" t="n">
         <v>100</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>score</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Gap</t>
+          <t>Greenwashing</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>FP2635</t>
+          <t>Risk score</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>57.1/100</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Non-Performing Loans (Portfolio at Risk): 30 Days</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr"/>
+          <t>Moderate Risk</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="n">
+        <v>57.1</v>
+      </c>
+      <c r="F28" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>risk</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2892,20 +2966,26 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>OD4091</t>
+          <t>Coverage</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Social and Environmental Targets</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr"/>
+          <t>47.1%</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" s="5" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="F29" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2915,7 +2995,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>OD8350</t>
+          <t>FP2635</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2925,7 +3005,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Client Model</t>
+          <t>Non-Performing Loans (Portfolio at Risk): 30 Days</t>
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
@@ -2938,7 +3018,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>OI1582</t>
+          <t>OD4091</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2948,7 +3028,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Wage Equity</t>
+          <t>Social and Environmental Targets</t>
         </is>
       </c>
       <c r="G31" t="inlineStr"/>
@@ -2961,7 +3041,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>OI4724</t>
+          <t>OD8350</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2971,7 +3051,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Workers Earning a Living Wage or Higher</t>
+          <t>Client Model</t>
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
@@ -2984,7 +3064,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>OI4732</t>
+          <t>OI1582</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2994,7 +3074,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Social and Environmental Performance Reporting</t>
+          <t>Wage Equity</t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
@@ -3007,7 +3087,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>OI4753</t>
+          <t>OI4724</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -3017,7 +3097,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Client Protection Policy</t>
+          <t>Workers Earning a Living Wage or Higher</t>
         </is>
       </c>
       <c r="G34" t="inlineStr"/>
@@ -3030,7 +3110,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>OI5049</t>
+          <t>OI4732</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -3040,7 +3120,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Client Feedback System</t>
+          <t>Social and Environmental Performance Reporting</t>
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
@@ -3053,7 +3133,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>PI9319</t>
+          <t>OI4753</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -3063,7 +3143,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Client Retention Rate</t>
+          <t>Client Protection Policy</t>
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
@@ -3076,27 +3156,20 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>FP4761</t>
+          <t>OI5049</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>32%</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Revenue Growth</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="n">
-        <v>32</v>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
+          <t>Client Feedback System</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3106,21 +3179,18 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>OI1075</t>
+          <t>PI9319</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Board of Directors: Total</t>
-        </is>
-      </c>
-      <c r="E38" s="5" t="n">
-        <v>7</v>
+          <t>Client Retention Rate</t>
+        </is>
       </c>
       <c r="G38" t="inlineStr"/>
     </row>
@@ -3132,25 +3202,25 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>OI1479</t>
+          <t>FP4761</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>120 tCO2e</t>
+          <t>32%</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Greenhouse Gas Emissions: Total</t>
+          <t>Revenue Growth</t>
         </is>
       </c>
       <c r="E39" s="5" t="n">
-        <v>120</v>
+        <v>32</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>tCO2e</t>
+          <t>%</t>
         </is>
       </c>
     </row>
@@ -3162,21 +3232,21 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>OI1571</t>
+          <t>OI1075</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>7</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Full-time Employees: Female Managers</t>
+          <t>Board of Directors: Total</t>
         </is>
       </c>
       <c r="E40" s="5" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="G40" t="inlineStr"/>
     </row>
@@ -3188,21 +3258,21 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>OI4112</t>
+          <t>OI1479</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>80 tCO2e</t>
+          <t>120 tCO2e</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Greenhouse Gas Emissions: Direct (Scope 1)</t>
+          <t>Greenhouse Gas Emissions: Total</t>
         </is>
       </c>
       <c r="E41" s="5" t="n">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -3218,21 +3288,21 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>OI6213</t>
+          <t>OI1571</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>12</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Full-time Employees: Female</t>
+          <t>Full-time Employees: Female Managers</t>
         </is>
       </c>
       <c r="E42" s="5" t="n">
-        <v>85</v>
+        <v>12</v>
       </c>
       <c r="G42" t="inlineStr"/>
     </row>
@@ -3244,23 +3314,27 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>OI8869</t>
+          <t>OI4112</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>80 tCO2e</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Permanent Employees: Total</t>
+          <t>Greenhouse Gas Emissions: Direct (Scope 1)</t>
         </is>
       </c>
       <c r="E43" s="5" t="n">
-        <v>180</v>
-      </c>
-      <c r="G43" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>tCO2e</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3270,67 +3344,73 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>PI4060</t>
+          <t>OI6213</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>45,000</t>
+          <t>85</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Client Individuals: Total</t>
+          <t>Full-time Employees: Female</t>
         </is>
       </c>
       <c r="E44" s="5" t="n">
-        <v>45000</v>
+        <v>85</v>
       </c>
       <c r="G44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Claim</t>
+          <t>Gap</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>outcome</t>
+          <t>OI8869</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>We serve 45,000 clients (PI4060: 45,000), 68% of them women.</t>
+          <t>180</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>metrics: PI4060</t>
-        </is>
+          <t>Permanent Employees: Total</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="n">
+        <v>180</v>
       </c>
       <c r="G45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Claim</t>
+          <t>Gap</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>outcome</t>
+          <t>PI4060</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Revenue grew 32% last year (FP4761: 32%).</t>
+          <t>45,000</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t xml:space="preserve">metrics: </t>
-        </is>
+          <t>Client Individuals: Total</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="n">
+        <v>45000</v>
       </c>
       <c r="G46" t="inlineStr"/>
     </row>
@@ -3347,12 +3427,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Portfolio at risk over 30 days is 3.1%.</t>
+          <t>We serve 45,000 clients (PI4060: 45,000), 68% of them women.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t xml:space="preserve">metrics: </t>
+          <t>metrics: PI4060</t>
         </is>
       </c>
       <c r="G47" t="inlineStr"/>
@@ -3370,18 +3450,87 @@
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
+          <t>We employ 180 permanent staff (OI8869: 180), including 85 women (OI6213: 85) and 12 female managers (OI1571: 12).</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>metrics: OI8869</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>outcome</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Revenue grew 32% last year (FP4761: 32%).</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">metrics: </t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>outcome</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Portfolio at risk over 30 days is 3.1%.</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">metrics: </t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>outcome</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
           <t>Our own footprint is 120 tCO2e (OI1479: 120 tCO2e), of which 80 tCO2e are direct Scope 1 emissions (OI4112: 80 tCO2e).</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>metrics: OI1479</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr"/>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>metrics: OI1479,OI4112</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G48"/>
+  <autoFilter ref="A1:G51"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3392,7 +3541,830 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:F36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AI disclosure</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Automated analysis: produced by rules and a deterministic scoring model; no generative AI was used. 3 of 21 scores are estimated from document text rather than reported metrics. Review before relying on it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Claim extraction</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Score calculation</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>deterministic</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Metric / SDG tagging</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Narrative drafting</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Generative AI used</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Scores estimated from text</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>3 of 21</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Human review</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>not recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Regulation</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>EU AI Act Art 50 transparency (Regulation (EU) 2024/1689 as amended by Regulation (EU) 2026/1744)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Figure</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Stage</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Estimated</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Five Dimensions: what</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>calculation</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>deterministic</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>evidence: partial</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Five Dimensions: who</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>calculation</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>deterministic</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>evidence: evidence-based</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Five Dimensions: how much</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>calculation</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>deterministic</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>evidence: estimated</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Five Dimensions: contribution</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>calculation</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>deterministic</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>evidence: estimated</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Five Dimensions: risk</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>calculation</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>deterministic</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>evidence: estimated</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>SDG 1 alignment</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>calculation</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>deterministic</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>basis: core_set</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>SDG 2 alignment</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>calculation</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>deterministic</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>basis: core_set</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>SDG 5 alignment</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>calculation</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>deterministic</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>basis: core_set</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>SDG 8 alignment</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>calculation</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>deterministic</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>basis: core_set</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>SDG 9 alignment</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>calculation</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>deterministic</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>basis: core_set</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>SDG 10 alignment</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>calculation</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>deterministic</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>basis: core_set</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>SDG 6 alignment</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>calculation</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>deterministic</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>basis: core_set</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>SDG 3 alignment</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>calculation</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>deterministic</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>basis: core_set</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>SDG 16 alignment</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>calculation</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>deterministic</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>basis: core_set</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>SDG 7 alignment</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>calculation</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>deterministic</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>basis: core_set</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>SDG 15 alignment</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>calculation</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>deterministic</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>basis: core_set</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>SDG 13 alignment</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>calculation</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>deterministic</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>basis: core_set</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>SDG 4 alignment</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>calculation</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>deterministic</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>basis: core_set</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>SDG 11 alignment</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>calculation</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>deterministic</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>basis: core_set</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>SDG 12 alignment</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>calculation</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>deterministic</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>basis: core_set</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>SDG 14 alignment</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>calculation</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>deterministic</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>basis: core_set</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>5 impact claims</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>IRIS+ / SDG mapping of claims</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>tagging</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A13:F36"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3431,31 +4403,31 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Scores (1–5) for What, Who, How Much, Contribution and Risk come from reported metrics where available and from document text otherwise.</t>
+          <t>Each dimension scores 1–5: coverage of the theme's IRIS+ reference set × 4.5 + 0.5 when any metric is reported, plus up to 0.5 for extra metrics. A dimension stays at or below 2.5 until 3 metrics hit its reference set; text-only inference is clamped to 0.5–2.5. Grades: A ≥ 4.5, B+ ≥ 3.5, B ≥ 3.0, B- ≥ 2.5, C+ ≥ 2.0, C ≥ 1.5, D ≥ 1.0.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SDGs</t>
+          <t>5D penalties</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Scores (0–100) combine goal-specific metric coverage and inference from the business and impact themes; cross-cutting metrics count at reduced weight. 'Material' marks goals the business model directly drives.</t>
+          <t>Risk loses 0.3 per unmitigated adverse impact (max 1.5) and 0.5 per exclusion flag (max 1.0).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Gap analysis</t>
+          <t>SDGs</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Coverage is the share of the sector's IRIS+ core metric set the company reports.</t>
+          <t>Each goal scores 0–100: up to 60 points from goal-specific metric coverage (metrics tagged to 6+ goals count at 0.4 weight), up to 25 from the business description and up to 15 from impact themes. High confidence needs ≥50 points and at least one goal-specific metric. Own-footprint metrics (OI4112, OI9604, OI1479, OI1697) are disclosure, not contribution, and count at the reduced weight.</t>
         </is>
       </c>
     </row>
@@ -3467,48 +4439,84 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Risk (0–100) weights claim–metric gaps (30%), missing negative impacts (20%), vague language (20%), selective reporting (15%) and lack of verification (15%). 60+ is flagged for review.</t>
+          <t>Risk (0–100) weights claim–metric gaps (30%), missing negative impacts (20%), vague language (20%), selective reporting (15%) and lack of verification (15%). Bands: ≤20 Genuine Impact Leader; ≤40 Substantive with Gaps; ≤60 Moderate Risk; ≤80 High Risk; ≤100 Probable Greenwashing.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>IC gate</t>
+          <t>Version</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Applies the fund thesis thresholds. Failures caused by missing data are reported as insufficient evidence, not as a negative finding.</t>
+          <t>Methodology v1.1.0 · config 8fabf9b5a7e2 (effective 2026-10-07).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Standards</t>
+          <t>Gap analysis</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>IRIS+ 5.3c catalog, IMP Five Dimensions, UN SDG framework (17 goals, 169 targets).</t>
+          <t>Coverage is the share of the sector's IRIS+ core metric set the company reports.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>IC gate</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Applies the fund thesis thresholds. Failures caused by missing data are reported as insufficient evidence, not as a negative finding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Standards</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>IRIS+ 5.3c catalog, IMP Five Dimensions, UN SDG framework (17 goals, 169 targets).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Schema</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Export schema version 1.0. Numeric cells are numbers; '—' marks values that were not reported.</t>
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>AI use</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Automated analysis: produced by rules and a deterministic scoring model; no generative AI was used. 3 of 21 scores are estimated from document text rather than reported metrics. Review before relying on it.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B9"/>
+  <autoFilter ref="A1:B12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
release: 0.17.1 — report styling pass across every deliverable
- fix self-referencing --warning token (memo/DD warning styles rendered black)
- IC memo: needs-data tones, evidence-to-collect callout, recommendation tone, gate tile;
  real Word output (runs, tables, house style, page numbers); DD .docx shares the style
- decision report: named metrics in ledger, non-wrapping pills, over-threshold greenwashing
  bars (warning + marker + legend), merged duplicate actions, named IDs, sorted goals
- shared CSS: flat token bars, status-only tile accents, nowrap pills, callout lists;
  grade colours on ink tokens (AA); DD tags humanized; portal centred + tokenized
- demo and screenshots regenerated; visual QA covers engagements

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo/brightpath_finance/brightpath_finance_data.xlsx
+++ b/demo/brightpath_finance/brightpath_finance_data.xlsx
@@ -527,7 +527,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-07T00:37:40Z</t>
+          <t>2026-10-07T00:55:04Z</t>
         </is>
       </c>
     </row>
@@ -2151,7 +2151,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-10-07T00:37:40Z</t>
+          <t>2026-10-07T00:55:04Z</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>

</xml_diff>

<commit_message>
fix: screenshot review: version strings, evidence ledger print, tidy images
- /version printed "OpenHarness 0.1.6"; now the installed Impact Vision
  version. OpenAI client User-Agent no longer hard-codes 0.14.0.
- Evidence ledger gets fixed column widths (claim column no longer
  collapses in the PDF); masthead date stays on one line on mobile.
- 5D notes pluralise correctly and read "N reported · X of Y reference".
- zh language note mentions DD questions shown in the original.
- Remove 4 unused images; regenerate demo + all screenshots (web chat
  shows v0.17.1); height-capped captures cut at a row boundary.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo/brightpath_finance/brightpath_finance_data.xlsx
+++ b/demo/brightpath_finance/brightpath_finance_data.xlsx
@@ -527,7 +527,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-07T00:55:04Z</t>
+          <t>2026-10-07T01:08:43Z</t>
         </is>
       </c>
     </row>
@@ -733,7 +733,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Reporting 2 metrics (0 theme-specific, 14 available)</t>
+          <t>2 metrics reported · 0 of 14 reference metrics</t>
         </is>
       </c>
     </row>
@@ -754,7 +754,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Reporting 5 metrics (0 theme-specific, 6 available)</t>
+          <t>5 metrics reported · 0 of 6 reference metrics</t>
         </is>
       </c>
     </row>
@@ -817,7 +817,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Estimated from sector/description (4 metrics available to track)</t>
+          <t>Estimated from sector/description · 4 reference metrics to track</t>
         </is>
       </c>
     </row>
@@ -2151,7 +2151,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-10-07T00:55:04Z</t>
+          <t>2026-10-07T01:08:43Z</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -2250,7 +2250,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Reporting 2 metrics (0 theme-specific, 14 available)</t>
+          <t>2 metrics reported · 0 of 14 reference metrics</t>
         </is>
       </c>
       <c r="E7" s="5" t="n">
@@ -2283,7 +2283,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Reporting 5 metrics (0 theme-specific, 6 available)</t>
+          <t>5 metrics reported · 0 of 6 reference metrics</t>
         </is>
       </c>
       <c r="E8" s="5" t="n">
@@ -2382,7 +2382,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Estimated from sector/description (4 metrics available to track)</t>
+          <t>Estimated from sector/description · 4 reference metrics to track</t>
         </is>
       </c>
       <c r="E11" s="5" t="n">

</xml_diff>

<commit_message>
feat: portfolio home shows stage, expected impact and evidence; totals in natural units (v8 W1.10, W3.1)
Portfolio vs pipeline from the company record; expected impact summed per
unit across invested companies (or the pipeline before any investment),
never an average of ordinal scores; per-company Impact P50 and Evidence
columns in the heat-map.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo/brightpath_finance/brightpath_finance_data.xlsx
+++ b/demo/brightpath_finance/brightpath_finance_data.xlsx
@@ -527,7 +527,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-08T16:14:47Z</t>
+          <t>2026-10-08T19:53:06Z</t>
         </is>
       </c>
     </row>
@@ -2151,7 +2151,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-10-08T16:14:47Z</t>
+          <t>2026-10-08T19:53:06Z</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>

</xml_diff>

<commit_message>
release: 0.18.0 "Measured" (roadmap v8, first pass of Waves 1–5)
- Excel/CSV KPI import (W3.5): spreadsheets dropped with a deck become
  reported metrics; series kept, unmatched labels listed.
- Deprecated roadmap_v2 / questionnaire_v2 / frameworks.sfdr_v2 shims
  removed (tests import the real modules).
- README describes expected impact and the three-state verdict; CHANGELOG
  0.18.0; roadmap v8 progress (done vs still to do); CLAUDE.md current
  release + new modules; regenerated demo and screenshots.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo/brightpath_finance/brightpath_finance_data.xlsx
+++ b/demo/brightpath_finance/brightpath_finance_data.xlsx
@@ -527,7 +527,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-08T19:53:06Z</t>
+          <t>2026-10-08T20:03:50Z</t>
         </is>
       </c>
     </row>
@@ -2151,7 +2151,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-10-08T19:53:06Z</t>
+          <t>2026-10-08T20:03:50Z</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>

</xml_diff>

<commit_message>
release: 0.19.0 Connected (roadmap v8, second pass)
CHANGELOG entry, version bump, roadmap progress with the held-out
baseline and its known misses, CLAUDE.md module map, and the demo bundle
regenerated on 0.19.0 (PDFs included). The enterprise-contribution tile
now quotes its strongest evidence (comparison group before baseline).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo/brightpath_finance/brightpath_finance_data.xlsx
+++ b/demo/brightpath_finance/brightpath_finance_data.xlsx
@@ -527,7 +527,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-08T20:03:50Z</t>
+          <t>2026-10-09T05:02:04Z</t>
         </is>
       </c>
     </row>
@@ -2151,7 +2151,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-10-08T20:03:50Z</t>
+          <t>2026-10-09T05:02:04Z</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>

</xml_diff>

<commit_message>
release: 0.19.1 Connected (roadmap v8, completion pass)
CHANGELOG [0.19.1] collects the work after 0.19.0: connectors,
calibration study kit and corpus, agent evals, reviewer sign-off, China
MoF profile, PCAF Dec-2025 update, HKFRS S1 gap tool and the Scope 3
method flag. README tags these capabilities (v0.19) inline in the
Frameworks table; version bumped in pyproject, CLAUDE.md and the
roadmap; demo bundle regenerated on 0.19.1.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo/brightpath_finance/brightpath_finance_data.xlsx
+++ b/demo/brightpath_finance/brightpath_finance_data.xlsx
@@ -527,7 +527,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-09T05:02:04Z</t>
+          <t>2026-10-09T09:37:49Z</t>
         </is>
       </c>
     </row>
@@ -2151,7 +2151,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-10-09T05:02:04Z</t>
+          <t>2026-10-09T09:37:49Z</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>

</xml_diff>